<commit_message>
Fixing some section of audit Section 2_3
</commit_message>
<xml_diff>
--- a/audit/docker_benchmark_reports/192.168.1.8_section2_3.xlsx
+++ b/audit/docker_benchmark_reports/192.168.1.8_section2_3.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Chart" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detailed Results'!$B$1:$H$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detailed Results'!$B$1:$H$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -91,7 +91,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="009C2B26"/>
+      <color rgb="001A4E8A"/>
       <sz val="10"/>
     </font>
     <font>
@@ -100,8 +100,20 @@
       <color rgb="001A6E2E"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009C2B26"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00555555"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -135,7 +147,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FAD7D5"/>
+        <fgColor rgb="00D0E8FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -146,6 +158,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D6F4DC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FAD7D5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8E8E8"/>
       </patternFill>
     </fill>
   </fills>
@@ -175,7 +197,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -222,6 +244,12 @@
     <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -238,6 +266,12 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -745,19 +779,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:J19"/>
+  <dimension ref="B1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="5" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="1" customWidth="1" min="9" max="9"/>
-    <col width="1" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -771,7 +796,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Daemon Configuration &amp; Files  |  Host: Docker-2204-DA-AUTO  |  OS: Ubuntu 22.04  |  2026-05-18T01:55:11Z</t>
+          <t>Daemon Configuration &amp; Files  |  Host: Docker-2204-DA-AUTO  |  Docker:   |  OS: Ubuntu 22.04  |  2026-05-18T05:21:16Z</t>
         </is>
       </c>
     </row>
@@ -800,27 +825,25 @@
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="B6" s="4" t="n">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" ht="12" customHeight="1"/>
+        <v>13</v>
+      </c>
+    </row>
     <row r="8" ht="28" customHeight="1">
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Compliance:  █████████████░░░░░░░  66.7%  (6 / 9 passed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="12" customHeight="1"/>
+          <t xml:space="preserve">  Compliance:  ███████████░░░░░░░░░  56.1%  (23 / 41 passed)</t>
+        </is>
+      </c>
+    </row>
     <row r="10" ht="22" customHeight="1">
       <c r="B10" s="9" t="inlineStr">
         <is>
@@ -851,17 +874,17 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Ensure TLS Authentication is enabled</t>
+          <t>Run the Docker daemon as a non-root user, if possible</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>TLS Authentication is NOT correctly enabled in daemon.json</t>
+          <t>Manual check required. Verify if Docker is running as non-root user. Standard Docker installations run as root. Rootless mode requires manual setup.</t>
         </is>
       </c>
     </row>
@@ -873,7 +896,7 @@
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>Ensure logging is configured correctly</t>
+          <t>Ensure network traffic is restricted between containers on the default bridge</t>
         </is>
       </c>
       <c r="F12" s="15" t="inlineStr">
@@ -883,7 +906,7 @@
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
-          <t>Logging is configured correctly with json-file driver, 10m max-size, 3 max-file.</t>
+          <t>ICC (inter-container communication) is disabled.</t>
         </is>
       </c>
     </row>
@@ -895,17 +918,17 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>Ensure User Namespace Remapping is enabled</t>
-        </is>
-      </c>
-      <c r="F13" s="12" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Ensure the logging level is set to 'info'</t>
+        </is>
+      </c>
+      <c r="F13" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>User Namespace Remapping is NOT enabled or subuid/subgid files missing</t>
+          <t>Logging level is set to info.</t>
         </is>
       </c>
     </row>
@@ -917,17 +940,17 @@
       </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
-          <t>Ensure Legacy Registry is disabled</t>
-        </is>
-      </c>
-      <c r="F14" s="12" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Ensure Docker is allowed to make changes to iptables</t>
+        </is>
+      </c>
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
-          <t>Legacy Registry is NOT disabled</t>
+          <t>Docker is configured to manage iptables.</t>
         </is>
       </c>
     </row>
@@ -939,7 +962,7 @@
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>Ensure Live Restore is enabled</t>
+          <t>Ensure insecure registries are not used</t>
         </is>
       </c>
       <c r="F15" s="15" t="inlineStr">
@@ -949,19 +972,19 @@
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
-          <t>Live Restore is enabled - containers continue running if Docker daemon stops.</t>
+          <t>No insecure registries configured.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="26" customHeight="1">
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>3.1.1</t>
+          <t>2.6</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
-          <t>Ensure /var/run/docker.sock ownership and permissions are correct</t>
+          <t>Ensure aufs storage driver is not used</t>
         </is>
       </c>
       <c r="F16" s="15" t="inlineStr">
@@ -971,19 +994,19 @@
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>Docker socket ownership and permissions are correct (root:docker 0660).</t>
+          <t>Storage driver is  (not aufs).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>3.1.2</t>
+          <t>2.7</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Ensure /etc/docker/daemon.json ownership and permissions are correct</t>
+          <t>Ensure devicemapper storage driver is not used</t>
         </is>
       </c>
       <c r="F17" s="15" t="inlineStr">
@@ -993,19 +1016,19 @@
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
-          <t>daemon.json ownership and permissions are correct (root:root 0644).</t>
+          <t>Storage driver is  (not devicemapper).</t>
         </is>
       </c>
     </row>
     <row r="18" ht="26" customHeight="1">
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>3.1.3</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
-          <t>Ensure docker.service ownership and permissions are correct</t>
+          <t>Ensure TLS authentication for Docker daemon is configured</t>
         </is>
       </c>
       <c r="F18" s="15" t="inlineStr">
@@ -1015,19 +1038,19 @@
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>docker.service ownership and permissions are correct (root:root 0644).</t>
+          <t>TLS authentication is enabled with tls and tlsverify configured.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="26" customHeight="1">
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>3.1.4</t>
+          <t>2.9</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>Ensure /var/lib/docker ownership and permissions are correct</t>
+          <t>Ensure the default ulimit is configured appropriately</t>
         </is>
       </c>
       <c r="F19" s="15" t="inlineStr">
@@ -1037,62 +1060,895 @@
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>/var/lib/docker ownership and permissions are correct (root:root 0710).</t>
+          <t>Default ulimits are configured in daemon.json.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>Enable user namespace support</t>
+        </is>
+      </c>
+      <c r="F20" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G20" s="14" t="inlineStr">
+        <is>
+          <t>User namespace remapping is enabled with default profile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Ensure the default cgroup usage has been confirmed</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>Cgroup driver: 
+INFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>2.12</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>Ensure base device size is not changed until needed</t>
+        </is>
+      </c>
+      <c r="F22" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G22" s="14" t="inlineStr">
+        <is>
+          <t>PASS: No custom base size</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>2.13</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>Ensure that authorization for Docker client commands is enabled</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>Authorization plugins are NOT configured. Docker commands are not audited/controlled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>2.14</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>Ensure centralized and remote logging is configured</t>
+        </is>
+      </c>
+      <c r="F24" s="16" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>Centralized logging is NOT configured. Logs may be lost if host fails.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>2.15</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>Ensure containers are restricted from acquiring new privileges</t>
+        </is>
+      </c>
+      <c r="F25" s="16" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>no-new-privileges is NOT set. Containers can escalate privileges via setuid binaries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>2.16</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>Ensure live restore is enabled</t>
+        </is>
+      </c>
+      <c r="F26" s="16" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G26" s="14" t="inlineStr">
+        <is>
+          <t>Live restore is NOT enabled. Containers stop when Docker daemon restarts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="26" customHeight="1">
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>2.17</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>Ensure Userland Proxy is Disabled</t>
+        </is>
+      </c>
+      <c r="F27" s="16" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G27" s="11" t="inlineStr">
+        <is>
+          <t>Userland proxy is enabled. This can cause performance issues and port conflicts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="26" customHeight="1">
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>2.18</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>Ensure that a daemon-wide custom seccomp profile is applied if appropriate</t>
+        </is>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="G28" s="14" t="inlineStr">
+        <is>
+          <t>INFO: Using default seccomp profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="26" customHeight="1">
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>2.19</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>Ensure that experimental features are not implemented in production</t>
+        </is>
+      </c>
+      <c r="F29" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G29" s="11" t="inlineStr">
+        <is>
+          <t>Experimental features are NOT enabled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="26" customHeight="1">
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>Ensure that the docker.service file ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="F30" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t>docker.service ownership is correct (root:root).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="26" customHeight="1">
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>Ensure that docker.service file permissions are appropriately set</t>
+        </is>
+      </c>
+      <c r="F31" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>docker.service permissions are correct (644 or 444).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="26" customHeight="1">
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>Ensure that docker.socket file ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="F32" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G32" s="14" t="inlineStr">
+        <is>
+          <t>docker.socket ownership is correct (root:root).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="26" customHeight="1">
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="inlineStr">
+        <is>
+          <t>Ensure that docker.socket file permissions are set to 644 or more restrictive</t>
+        </is>
+      </c>
+      <c r="F33" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="inlineStr">
+        <is>
+          <t>docker.socket permissions are correct (644 or 444).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="26" customHeight="1">
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="D34" s="14" t="inlineStr">
+        <is>
+          <t>Ensure that registry certificate file ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="F34" s="17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="G34" s="14" t="inlineStr">
+        <is>
+          <t>No registry certificates found in /etc/docker/certs.d.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="26" customHeight="1">
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>3.6</t>
+        </is>
+      </c>
+      <c r="D35" s="11" t="inlineStr">
+        <is>
+          <t>Ensure that registry certificate file permissions are set to 444 or more restrictively</t>
+        </is>
+      </c>
+      <c r="F35" s="17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="G35" s="11" t="inlineStr">
+        <is>
+          <t>No registry certificates found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="26" customHeight="1">
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
+      <c r="D36" s="14" t="inlineStr">
+        <is>
+          <t>Ensure that TLS CA certificate ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="F36" s="17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="G36" s="14" t="inlineStr">
+        <is>
+          <t>No TLS CA certificates found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="26" customHeight="1">
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>3.8</t>
+        </is>
+      </c>
+      <c r="D37" s="11" t="inlineStr">
+        <is>
+          <t>Ensure that TLS CA certificate permissions are set to 444 or more restrictively</t>
+        </is>
+      </c>
+      <c r="F37" s="17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="G37" s="11" t="inlineStr">
+        <is>
+          <t>No TLS CA certificates found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="26" customHeight="1">
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>3.9</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="inlineStr">
+        <is>
+          <t>Ensure that Docker server certificate file ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="F38" s="17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="G38" s="14" t="inlineStr">
+        <is>
+          <t>No Docker server certificates found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="26" customHeight="1">
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="inlineStr">
+        <is>
+          <t>Ensure that Docker server certificate file permissions are set to 444 or more restrictively</t>
+        </is>
+      </c>
+      <c r="F39" s="17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="G39" s="11" t="inlineStr">
+        <is>
+          <t>No Docker server certificates found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="26" customHeight="1">
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>3.11</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr">
+        <is>
+          <t>Ensure that the Docker server certificate key file ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="F40" s="17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="G40" s="14" t="inlineStr">
+        <is>
+          <t>No Docker server keys found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="26" customHeight="1">
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>3.12</t>
+        </is>
+      </c>
+      <c r="D41" s="11" t="inlineStr">
+        <is>
+          <t>Ensure that the Docker server certificate key file permissions are set to 400</t>
+        </is>
+      </c>
+      <c r="F41" s="17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="G41" s="11" t="inlineStr">
+        <is>
+          <t>No Docker server keys found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="26" customHeight="1">
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>3.13</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="inlineStr">
+        <is>
+          <t>Ensure that the Docker socket file ownership is set to root:docker</t>
+        </is>
+      </c>
+      <c r="F42" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G42" s="14" t="inlineStr">
+        <is>
+          <t>Docker socket ownership is correct (root:docker).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="26" customHeight="1">
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>3.14</t>
+        </is>
+      </c>
+      <c r="D43" s="11" t="inlineStr">
+        <is>
+          <t>Ensure that the Docker socket file permissions are set to 660 or more restrictively</t>
+        </is>
+      </c>
+      <c r="F43" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G43" s="11" t="inlineStr">
+        <is>
+          <t>Docker socket permissions are correct (660 or more restrictive).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="26" customHeight="1">
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>3.15</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="inlineStr">
+        <is>
+          <t>Ensure that the daemon.json file ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="F44" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G44" s="14" t="inlineStr">
+        <is>
+          <t>daemon.json ownership is correct (root:root).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="26" customHeight="1">
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>3.16</t>
+        </is>
+      </c>
+      <c r="D45" s="11" t="inlineStr">
+        <is>
+          <t>Ensure that daemon.json file permissions are set to 644 or more restrictive</t>
+        </is>
+      </c>
+      <c r="F45" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr">
+        <is>
+          <t>daemon.json permissions are correct (644 or more restrictive).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="26" customHeight="1">
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>3.17</t>
+        </is>
+      </c>
+      <c r="D46" s="14" t="inlineStr">
+        <is>
+          <t>Ensure that the /etc/default/docker file ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="F46" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G46" s="14" t="inlineStr">
+        <is>
+          <t>/etc/default/docker ownership is correct (root:root).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="26" customHeight="1">
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>3.18</t>
+        </is>
+      </c>
+      <c r="D47" s="11" t="inlineStr">
+        <is>
+          <t>Ensure that the /etc/default/docker file permissions are set to 644 or more restrictively</t>
+        </is>
+      </c>
+      <c r="F47" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G47" s="11" t="inlineStr">
+        <is>
+          <t>/etc/default/docker permissions are correct (644 or more restrictive).</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="26" customHeight="1">
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>3.19</t>
+        </is>
+      </c>
+      <c r="D48" s="14" t="inlineStr">
+        <is>
+          <t>Ensure that the /etc/sysconfig/docker file permissions are set to 644 or more restrictively</t>
+        </is>
+      </c>
+      <c r="F48" s="17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="G48" s="14" t="inlineStr">
+        <is>
+          <t>/etc/sysconfig/docker does not exist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="26" customHeight="1">
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="D49" s="11" t="inlineStr">
+        <is>
+          <t>Ensure that the /etc/sysconfig/docker file ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="F49" s="17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="G49" s="11" t="inlineStr">
+        <is>
+          <t>/etc/sysconfig/docker does not exist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="26" customHeight="1">
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>3.21</t>
+        </is>
+      </c>
+      <c r="D50" s="14" t="inlineStr">
+        <is>
+          <t>Ensure that the Containerd socket file ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="F50" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G50" s="14" t="inlineStr">
+        <is>
+          <t>containerd socket ownership is correct (root:root).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="26" customHeight="1">
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>3.22</t>
+        </is>
+      </c>
+      <c r="D51" s="11" t="inlineStr">
+        <is>
+          <t>Ensure that the Containerd socket file permissions are set to 660 or more restrictively</t>
+        </is>
+      </c>
+      <c r="F51" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G51" s="11" t="inlineStr">
+        <is>
+          <t>containerd socket permissions are correct (660 or more restrictive).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="51">
+  <mergeCells count="179">
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="F39"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="G47:J47"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="F49"/>
+    <mergeCell ref="F14"/>
+    <mergeCell ref="G32:J32"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="G46:J46"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="G40:J40"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="F40"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="F12"/>
+    <mergeCell ref="F21"/>
+    <mergeCell ref="F51"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="G10:J10"/>
+    <mergeCell ref="F41"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="F35"/>
+    <mergeCell ref="F50"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="G34:J34"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="F31"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="F27"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="D10:E10"/>
+    <mergeCell ref="B25:C25"/>
     <mergeCell ref="D19:E19"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="G29:J29"/>
     <mergeCell ref="F6:G6"/>
-    <mergeCell ref="B8:J8"/>
-    <mergeCell ref="G16:J16"/>
     <mergeCell ref="B18:C18"/>
-    <mergeCell ref="F14"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="G44:J44"/>
+    <mergeCell ref="G22:J22"/>
+    <mergeCell ref="G31:J31"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D13:E13"/>
     <mergeCell ref="F5:G5"/>
     <mergeCell ref="G12:J12"/>
+    <mergeCell ref="F29"/>
     <mergeCell ref="F11"/>
-    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="F25"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="G48:J48"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="F15"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="F24"/>
+    <mergeCell ref="G38:J38"/>
+    <mergeCell ref="G45:J45"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="F32"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B1:J2"/>
+    <mergeCell ref="F26"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="G49:J49"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="G24:J24"/>
+    <mergeCell ref="F23"/>
+    <mergeCell ref="F38"/>
+    <mergeCell ref="G33:J33"/>
+    <mergeCell ref="F13"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="F43"/>
+    <mergeCell ref="G35:J35"/>
+    <mergeCell ref="F37"/>
+    <mergeCell ref="G16:J16"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="F44"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="B42:C42"/>
     <mergeCell ref="F19"/>
-    <mergeCell ref="F10"/>
+    <mergeCell ref="F34"/>
+    <mergeCell ref="F16"/>
     <mergeCell ref="G11:J11"/>
-    <mergeCell ref="F16"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="D17:E17"/>
-    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="G39:J39"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="F30"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="F20"/>
+    <mergeCell ref="F33"/>
+    <mergeCell ref="F42"/>
+    <mergeCell ref="G37:J37"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="G13:J13"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="G15:J15"/>
+    <mergeCell ref="F46"/>
+    <mergeCell ref="F28"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="F48"/>
+    <mergeCell ref="G51:J51"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="B8:J8"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="G41:J41"/>
+    <mergeCell ref="G50:J50"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="G43:J43"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="F10"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="G27:J27"/>
+    <mergeCell ref="G36:J36"/>
+    <mergeCell ref="G42:J42"/>
     <mergeCell ref="D16:E16"/>
     <mergeCell ref="G17:J17"/>
-    <mergeCell ref="F12"/>
-    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="D43:E43"/>
     <mergeCell ref="B10:C10"/>
-    <mergeCell ref="F15"/>
     <mergeCell ref="D18:E18"/>
     <mergeCell ref="G19:J19"/>
+    <mergeCell ref="F36"/>
     <mergeCell ref="F18"/>
-    <mergeCell ref="G10:J10"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="G13:J13"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B1:J2"/>
-    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="G28:J28"/>
+    <mergeCell ref="F45"/>
+    <mergeCell ref="D42:E42"/>
     <mergeCell ref="F17"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="G15:J15"/>
-    <mergeCell ref="F13"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="G30:J30"/>
+    <mergeCell ref="F47"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="F22"/>
     <mergeCell ref="G14:J14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1105,7 +1961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H10"/>
+  <dimension ref="B1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1156,330 +2012,1499 @@
       </c>
     </row>
     <row r="2" ht="44" customHeight="1">
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>2.1</t>
         </is>
       </c>
-      <c r="C2" s="17" t="inlineStr">
+      <c r="C2" s="19" t="inlineStr">
         <is>
           <t>Section 2 - Docker Daemon Configuration</t>
         </is>
       </c>
-      <c r="D2" s="17" t="inlineStr">
-        <is>
-          <t>Ensure TLS Authentication is enabled</t>
-        </is>
-      </c>
-      <c r="E2" s="18" t="inlineStr">
+      <c r="D2" s="19" t="inlineStr">
+        <is>
+          <t>Run the Docker daemon as a non-root user, if possible</t>
+        </is>
+      </c>
+      <c r="E2" s="20" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="F2" s="19" t="inlineStr">
+        <is>
+          <t>Manual check required. Verify if Docker is running as non-root user. Standard Docker installations run as root. Rootless mode requires manual setup.</t>
+        </is>
+      </c>
+      <c r="G2" s="19" t="inlineStr">
+        <is>
+          <t>Consider rootless Docker installation: https://docs.docker.com/engine/security/rootless/</t>
+        </is>
+      </c>
+      <c r="H2" s="19" t="inlineStr">
+        <is>
+          <t>Manual check - review with: ps -ef | grep dockerd</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="44" customHeight="1">
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="C3" s="22" t="inlineStr">
+        <is>
+          <t>Section 2 - Docker Daemon Configuration</t>
+        </is>
+      </c>
+      <c r="D3" s="22" t="inlineStr">
+        <is>
+          <t>Ensure network traffic is restricted between containers on the default bridge</t>
+        </is>
+      </c>
+      <c r="E3" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F3" s="22" t="inlineStr">
+        <is>
+          <t>ICC (inter-container communication) is disabled.</t>
+        </is>
+      </c>
+      <c r="G3" s="22" t="inlineStr">
+        <is>
+          <t>Add "icc": false to /etc/docker/daemon.json and restart Docker.</t>
+        </is>
+      </c>
+      <c r="H3" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "icc": false,</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44" customHeight="1">
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="C4" s="19" t="inlineStr">
+        <is>
+          <t>Section 2 - Docker Daemon Configuration</t>
+        </is>
+      </c>
+      <c r="D4" s="19" t="inlineStr">
+        <is>
+          <t>Ensure the logging level is set to 'info'</t>
+        </is>
+      </c>
+      <c r="E4" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F4" s="19" t="inlineStr">
+        <is>
+          <t>Logging level is set to info.</t>
+        </is>
+      </c>
+      <c r="G4" s="19" t="inlineStr">
+        <is>
+          <t>Add "log-level": "info" to /etc/docker/daemon.json</t>
+        </is>
+      </c>
+      <c r="H4" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "log-level": "info",</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44" customHeight="1">
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="inlineStr">
+        <is>
+          <t>Section 2 - Docker Daemon Configuration</t>
+        </is>
+      </c>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
+          <t>Ensure Docker is allowed to make changes to iptables</t>
+        </is>
+      </c>
+      <c r="E5" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F5" s="22" t="inlineStr">
+        <is>
+          <t>Docker is configured to manage iptables.</t>
+        </is>
+      </c>
+      <c r="G5" s="22" t="inlineStr">
+        <is>
+          <t>Add "iptables": true to /etc/docker/daemon.json</t>
+        </is>
+      </c>
+      <c r="H5" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "iptables": true,</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>Section 2 - Docker Daemon Configuration</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>Ensure insecure registries are not used</t>
+        </is>
+      </c>
+      <c r="E6" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>No insecure registries configured.</t>
+        </is>
+      </c>
+      <c r="G6" s="19" t="inlineStr">
+        <is>
+          <t>Remove insecure registries from /etc/docker/daemon.json or set to empty array: []</t>
+        </is>
+      </c>
+      <c r="H6" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="44" customHeight="1">
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>Section 2 - Docker Daemon Configuration</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="inlineStr">
+        <is>
+          <t>Ensure aufs storage driver is not used</t>
+        </is>
+      </c>
+      <c r="E7" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F7" s="22" t="inlineStr">
+        <is>
+          <t>Storage driver is  (not aufs).</t>
+        </is>
+      </c>
+      <c r="G7" s="22" t="inlineStr">
+        <is>
+          <t>Change storage driver to overlay2 in /etc/docker/daemon.json: {"storage-driver": "overlay2"}</t>
+        </is>
+      </c>
+      <c r="H7" s="22" t="inlineStr"/>
+    </row>
+    <row r="8" ht="44" customHeight="1">
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>Section 2 - Docker Daemon Configuration</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>Ensure devicemapper storage driver is not used</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>Storage driver is  (not devicemapper).</t>
+        </is>
+      </c>
+      <c r="G8" s="19" t="inlineStr">
+        <is>
+          <t>Change storage driver to overlay2 in /etc/docker/daemon.json: {"storage-driver": "overlay2"}</t>
+        </is>
+      </c>
+      <c r="H8" s="19" t="inlineStr"/>
+    </row>
+    <row r="9" ht="44" customHeight="1">
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="inlineStr">
+        <is>
+          <t>Section 2 - Docker Daemon Configuration</t>
+        </is>
+      </c>
+      <c r="D9" s="22" t="inlineStr">
+        <is>
+          <t>Ensure TLS authentication for Docker daemon is configured</t>
+        </is>
+      </c>
+      <c r="E9" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F9" s="22" t="inlineStr">
+        <is>
+          <t>TLS authentication is enabled with tls and tlsverify configured.</t>
+        </is>
+      </c>
+      <c r="G9" s="22" t="inlineStr">
+        <is>
+          <t>Configure TLS in /etc/docker/daemon.json with "tls": true and "tlsverify": true. Ensure CA, server cert, and server key paths are correctly specified.</t>
+        </is>
+      </c>
+      <c r="H9" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "tls": true,
+    "tlsverify": true,</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="44" customHeight="1">
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>2.9</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>Section 2 - Docker Daemon Configuration</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Ensure the default ulimit is configured appropriately</t>
+        </is>
+      </c>
+      <c r="E10" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>Default ulimits are configured in daemon.json.</t>
+        </is>
+      </c>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>Configure default ulimits in /etc/docker/daemon.json: {"default-ulimits": {"nofile": {"Hard": 64000, "Name": "nofile", "Soft": 64000}}}</t>
+        </is>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>"default-ulimits": {</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="44" customHeight="1">
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="C11" s="22" t="inlineStr">
+        <is>
+          <t>Section 2 - Docker Daemon Configuration</t>
+        </is>
+      </c>
+      <c r="D11" s="22" t="inlineStr">
+        <is>
+          <t>Enable user namespace support</t>
+        </is>
+      </c>
+      <c r="E11" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F11" s="22" t="inlineStr">
+        <is>
+          <t>User namespace remapping is enabled with default profile.</t>
+        </is>
+      </c>
+      <c r="G11" s="22" t="inlineStr">
+        <is>
+          <t>Add "userns-remap": "default" to /etc/docker/daemon.json and restart Docker. Ensure /etc/subuid and /etc/subgid files exist with dockremap entries.</t>
+        </is>
+      </c>
+      <c r="H11" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "userns-remap": "default",</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="44" customHeight="1">
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>Section 2 - Docker Daemon Configuration</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Ensure the default cgroup usage has been confirmed</t>
+        </is>
+      </c>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>Cgroup driver: 
+INFO</t>
+        </is>
+      </c>
+      <c r="G12" s="19" t="inlineStr">
+        <is>
+          <t>Review cgroup driver configuration. Use cgroupfs or systemd consistently.</t>
+        </is>
+      </c>
+      <c r="H12" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+INFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="44" customHeight="1">
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>2.12</t>
+        </is>
+      </c>
+      <c r="C13" s="22" t="inlineStr">
+        <is>
+          <t>Section 2 - Docker Daemon Configuration</t>
+        </is>
+      </c>
+      <c r="D13" s="22" t="inlineStr">
+        <is>
+          <t>Ensure base device size is not changed until needed</t>
+        </is>
+      </c>
+      <c r="E13" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F13" s="22" t="inlineStr">
+        <is>
+          <t>PASS: No custom base size</t>
+        </is>
+      </c>
+      <c r="G13" s="22" t="inlineStr">
+        <is>
+          <t>Do not set dm.basesize unless required. Default is sufficient for most use cases.</t>
+        </is>
+      </c>
+      <c r="H13" s="22" t="inlineStr">
+        <is>
+          <t>PASS: No custom base size</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="44" customHeight="1">
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>2.13</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>Section 2 - Docker Daemon Configuration</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>Ensure that authorization for Docker client commands is enabled</t>
+        </is>
+      </c>
+      <c r="E14" s="24" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="F2" s="17" t="inlineStr">
-        <is>
-          <t>TLS Authentication is NOT correctly enabled in daemon.json</t>
-        </is>
-      </c>
-      <c r="G2" s="17" t="inlineStr">
-        <is>
-          <t>Configure TLS in /etc/docker/daemon.json with "tls": true and "tlsverify": true. Ensure CA, server cert, and server key paths are correctly specified.</t>
-        </is>
-      </c>
-      <c r="H2" s="17" t="inlineStr"/>
-    </row>
-    <row r="3" ht="44" customHeight="1">
-      <c r="B3" s="19" t="inlineStr">
-        <is>
-          <t>2.2</t>
-        </is>
-      </c>
-      <c r="C3" s="20" t="inlineStr">
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>Authorization plugins are NOT configured. Docker commands are not audited/controlled.</t>
+        </is>
+      </c>
+      <c r="G14" s="19" t="inlineStr">
+        <is>
+          <t>Add authorization plugins to /etc/docker/daemon.json: {"authorization-plugins": ["openpolicyagent/opa-docker-authz"]}</t>
+        </is>
+      </c>
+      <c r="H14" s="19" t="inlineStr"/>
+    </row>
+    <row r="15" ht="44" customHeight="1">
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <t>2.14</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="inlineStr">
         <is>
           <t>Section 2 - Docker Daemon Configuration</t>
         </is>
       </c>
-      <c r="D3" s="20" t="inlineStr">
-        <is>
-          <t>Ensure logging is configured correctly</t>
-        </is>
-      </c>
-      <c r="E3" s="21" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F3" s="20" t="inlineStr">
-        <is>
-          <t>Logging is configured correctly with json-file driver, 10m max-size, 3 max-file.</t>
-        </is>
-      </c>
-      <c r="G3" s="20" t="inlineStr">
-        <is>
-          <t>Configure logging in /etc/docker/daemon.json: {"log-driver": "json-file", "log-opts": {"max-size": "10m", "max-file": "3"}}</t>
-        </is>
-      </c>
-      <c r="H3" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  "log-driver": "json-file",
-    "max-size": "10m",
-    "max-file": "3"</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="44" customHeight="1">
-      <c r="B4" s="16" t="inlineStr">
-        <is>
-          <t>2.3</t>
-        </is>
-      </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="D15" s="22" t="inlineStr">
+        <is>
+          <t>Ensure centralized and remote logging is configured</t>
+        </is>
+      </c>
+      <c r="E15" s="24" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F15" s="22" t="inlineStr">
+        <is>
+          <t>Centralized logging is NOT configured. Logs may be lost if host fails.</t>
+        </is>
+      </c>
+      <c r="G15" s="22" t="inlineStr">
+        <is>
+          <t>Configure a centralized logging driver in /etc/docker/daemon.json: {"log-driver": "syslog", "log-opts": {"syslog-address": "tcp://192.168.0.42:12345"}}</t>
+        </is>
+      </c>
+      <c r="H15" s="22" t="inlineStr"/>
+    </row>
+    <row r="16" ht="44" customHeight="1">
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>2.15</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
         <is>
           <t>Section 2 - Docker Daemon Configuration</t>
         </is>
       </c>
-      <c r="D4" s="17" t="inlineStr">
-        <is>
-          <t>Ensure User Namespace Remapping is enabled</t>
-        </is>
-      </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>Ensure containers are restricted from acquiring new privileges</t>
+        </is>
+      </c>
+      <c r="E16" s="24" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="F4" s="17" t="inlineStr">
-        <is>
-          <t>User Namespace Remapping is NOT enabled or subuid/subgid files missing</t>
-        </is>
-      </c>
-      <c r="G4" s="17" t="inlineStr">
-        <is>
-          <t>Add "userns-remap": "default" to /etc/docker/daemon.json and restart Docker. Ensure /etc/subuid and /etc/subgid files exist.</t>
-        </is>
-      </c>
-      <c r="H4" s="17" t="inlineStr"/>
-    </row>
-    <row r="5" ht="44" customHeight="1">
-      <c r="B5" s="19" t="inlineStr">
-        <is>
-          <t>2.4</t>
-        </is>
-      </c>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>no-new-privileges is NOT set. Containers can escalate privileges via setuid binaries.</t>
+        </is>
+      </c>
+      <c r="G16" s="19" t="inlineStr">
+        <is>
+          <t>Add "no-new-privileges": true to /etc/docker/daemon.json</t>
+        </is>
+      </c>
+      <c r="H16" s="19" t="inlineStr"/>
+    </row>
+    <row r="17" ht="44" customHeight="1">
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>2.16</t>
+        </is>
+      </c>
+      <c r="C17" s="22" t="inlineStr">
         <is>
           <t>Section 2 - Docker Daemon Configuration</t>
         </is>
       </c>
-      <c r="D5" s="20" t="inlineStr">
-        <is>
-          <t>Ensure Legacy Registry is disabled</t>
-        </is>
-      </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="D17" s="22" t="inlineStr">
+        <is>
+          <t>Ensure live restore is enabled</t>
+        </is>
+      </c>
+      <c r="E17" s="24" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="F5" s="20" t="inlineStr">
-        <is>
-          <t>Legacy Registry is NOT disabled</t>
-        </is>
-      </c>
-      <c r="G5" s="20" t="inlineStr">
-        <is>
-          <t>Add "disable-legacy-registry": true to /etc/docker/daemon.json</t>
-        </is>
-      </c>
-      <c r="H5" s="20" t="inlineStr"/>
-    </row>
-    <row r="6" ht="44" customHeight="1">
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="F17" s="22" t="inlineStr">
+        <is>
+          <t>Live restore is NOT enabled. Containers stop when Docker daemon restarts.</t>
+        </is>
+      </c>
+      <c r="G17" s="22" t="inlineStr">
+        <is>
+          <t>Add "live-restore": true to /etc/docker/daemon.json</t>
+        </is>
+      </c>
+      <c r="H17" s="22" t="inlineStr"/>
+    </row>
+    <row r="18" ht="44" customHeight="1">
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>2.17</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
         <is>
           <t>Section 2 - Docker Daemon Configuration</t>
         </is>
       </c>
-      <c r="D6" s="17" t="inlineStr">
-        <is>
-          <t>Ensure Live Restore is enabled</t>
-        </is>
-      </c>
-      <c r="E6" s="21" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F6" s="17" t="inlineStr">
-        <is>
-          <t>Live Restore is enabled - containers continue running if Docker daemon stops.</t>
-        </is>
-      </c>
-      <c r="G6" s="17" t="inlineStr">
-        <is>
-          <t>Add "live-restore": true to /etc/docker/daemon.json and restart Docker.</t>
-        </is>
-      </c>
-      <c r="H6" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  "live-restore": true,</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="44" customHeight="1">
-      <c r="B7" s="19" t="inlineStr">
-        <is>
-          <t>3.1.1</t>
-        </is>
-      </c>
-      <c r="C7" s="20" t="inlineStr">
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>Ensure Userland Proxy is Disabled</t>
+        </is>
+      </c>
+      <c r="E18" s="24" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
+        <is>
+          <t>Userland proxy is enabled. This can cause performance issues and port conflicts.</t>
+        </is>
+      </c>
+      <c r="G18" s="19" t="inlineStr">
+        <is>
+          <t>Add "userland-proxy": false to /etc/docker/daemon.json</t>
+        </is>
+      </c>
+      <c r="H18" s="19" t="inlineStr"/>
+    </row>
+    <row r="19" ht="44" customHeight="1">
+      <c r="B19" s="21" t="inlineStr">
+        <is>
+          <t>2.18</t>
+        </is>
+      </c>
+      <c r="C19" s="22" t="inlineStr">
+        <is>
+          <t>Section 2 - Docker Daemon Configuration</t>
+        </is>
+      </c>
+      <c r="D19" s="22" t="inlineStr">
+        <is>
+          <t>Ensure that a daemon-wide custom seccomp profile is applied if appropriate</t>
+        </is>
+      </c>
+      <c r="E19" s="20" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="F19" s="22" t="inlineStr">
+        <is>
+          <t>INFO: Using default seccomp profile</t>
+        </is>
+      </c>
+      <c r="G19" s="22" t="inlineStr">
+        <is>
+          <t>If custom seccomp is needed, configure in daemon.json: {"seccomp-profile": "/etc/docker/seccomp/profile.json"}</t>
+        </is>
+      </c>
+      <c r="H19" s="22" t="inlineStr">
+        <is>
+          <t>INFO: Using default seccomp profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="44" customHeight="1">
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>2.19</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="inlineStr">
+        <is>
+          <t>Section 2 - Docker Daemon Configuration</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>Ensure that experimental features are not implemented in production</t>
+        </is>
+      </c>
+      <c r="E20" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>Experimental features are NOT enabled.</t>
+        </is>
+      </c>
+      <c r="G20" s="19" t="inlineStr">
+        <is>
+          <t>Remove or set "experimental": false in /etc/docker/daemon.json</t>
+        </is>
+      </c>
+      <c r="H20" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="44" customHeight="1">
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="C21" s="22" t="inlineStr">
         <is>
           <t>Section 3 - Docker Daemon Configuration Files</t>
         </is>
       </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>Ensure /var/run/docker.sock ownership and permissions are correct</t>
-        </is>
-      </c>
-      <c r="E7" s="21" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F7" s="20" t="inlineStr">
-        <is>
-          <t>Docker socket ownership and permissions are correct (root:docker 0660).</t>
-        </is>
-      </c>
-      <c r="G7" s="20" t="inlineStr">
-        <is>
-          <t>chown root:docker /var/run/docker.sock &amp;&amp; chmod 660 /var/run/docker.sock</t>
-        </is>
-      </c>
-      <c r="H7" s="20" t="inlineStr">
-        <is>
-          <t>root:docker mode=0660</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="44" customHeight="1">
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>3.1.2</t>
-        </is>
-      </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="D21" s="22" t="inlineStr">
+        <is>
+          <t>Ensure that the docker.service file ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="E21" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F21" s="22" t="inlineStr">
+        <is>
+          <t>docker.service ownership is correct (root:root).</t>
+        </is>
+      </c>
+      <c r="G21" s="22" t="inlineStr">
+        <is>
+          <t>chown root:root /usr/lib/systemd/system/docker.service</t>
+        </is>
+      </c>
+      <c r="H21" s="22" t="inlineStr">
+        <is>
+          <t>['root', AnsibleUndefined(hint=None, obj={'exists': False}, name='pw_name'), 'root']</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="44" customHeight="1">
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="inlineStr">
         <is>
           <t>Section 3 - Docker Daemon Configuration Files</t>
         </is>
       </c>
-      <c r="D8" s="17" t="inlineStr">
-        <is>
-          <t>Ensure /etc/docker/daemon.json ownership and permissions are correct</t>
-        </is>
-      </c>
-      <c r="E8" s="21" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F8" s="17" t="inlineStr">
-        <is>
-          <t>daemon.json ownership and permissions are correct (root:root 0644).</t>
-        </is>
-      </c>
-      <c r="G8" s="17" t="inlineStr">
-        <is>
-          <t>chown root:root /etc/docker/daemon.json &amp;&amp; chmod 644 /etc/docker/daemon.json</t>
-        </is>
-      </c>
-      <c r="H8" s="17" t="inlineStr">
-        <is>
-          <t>root:root mode=0644</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="44" customHeight="1">
-      <c r="B9" s="19" t="inlineStr">
-        <is>
-          <t>3.1.3</t>
-        </is>
-      </c>
-      <c r="C9" s="20" t="inlineStr">
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>Ensure that docker.service file permissions are appropriately set</t>
+        </is>
+      </c>
+      <c r="E22" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F22" s="19" t="inlineStr">
+        <is>
+          <t>docker.service permissions are correct (644 or 444).</t>
+        </is>
+      </c>
+      <c r="G22" s="19" t="inlineStr">
+        <is>
+          <t>chmod 644 /usr/lib/systemd/system/docker.service</t>
+        </is>
+      </c>
+      <c r="H22" s="19" t="inlineStr">
+        <is>
+          <t>['0644', AnsibleUndefined(hint=None, obj={'exists': False}, name='mode'), '0644']</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="44" customHeight="1">
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="C23" s="22" t="inlineStr">
         <is>
           <t>Section 3 - Docker Daemon Configuration Files</t>
         </is>
       </c>
-      <c r="D9" s="20" t="inlineStr">
-        <is>
-          <t>Ensure docker.service ownership and permissions are correct</t>
-        </is>
-      </c>
-      <c r="E9" s="21" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F9" s="20" t="inlineStr">
-        <is>
-          <t>docker.service ownership and permissions are correct (root:root 0644).</t>
-        </is>
-      </c>
-      <c r="G9" s="20" t="inlineStr">
-        <is>
-          <t>chown root:root /usr/lib/systemd/system/docker.service &amp;&amp; chmod 644</t>
-        </is>
-      </c>
-      <c r="H9" s="20" t="inlineStr">
-        <is>
-          <t>root:root mode=0644</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="44" customHeight="1">
-      <c r="B10" s="16" t="inlineStr">
-        <is>
-          <t>3.1.4</t>
-        </is>
-      </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="D23" s="22" t="inlineStr">
+        <is>
+          <t>Ensure that docker.socket file ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="E23" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F23" s="22" t="inlineStr">
+        <is>
+          <t>docker.socket ownership is correct (root:root).</t>
+        </is>
+      </c>
+      <c r="G23" s="22" t="inlineStr">
+        <is>
+          <t>chown root:root /usr/lib/systemd/system/docker.socket</t>
+        </is>
+      </c>
+      <c r="H23" s="22" t="inlineStr">
+        <is>
+          <t>['root', AnsibleUndefined(hint=None, obj={'exists': False}, name='pw_name'), 'root']</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="44" customHeight="1">
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="C24" s="19" t="inlineStr">
         <is>
           <t>Section 3 - Docker Daemon Configuration Files</t>
         </is>
       </c>
-      <c r="D10" s="17" t="inlineStr">
-        <is>
-          <t>Ensure /var/lib/docker ownership and permissions are correct</t>
-        </is>
-      </c>
-      <c r="E10" s="21" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F10" s="17" t="inlineStr">
-        <is>
-          <t>/var/lib/docker ownership and permissions are correct (root:root 0710).</t>
-        </is>
-      </c>
-      <c r="G10" s="17" t="inlineStr">
-        <is>
-          <t>chown root:root /var/lib/docker &amp;&amp; chmod 0710 /var/lib/docker</t>
-        </is>
-      </c>
-      <c r="H10" s="17" t="inlineStr">
-        <is>
-          <t>root:root mode=0710</t>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>Ensure that docker.socket file permissions are set to 644 or more restrictive</t>
+        </is>
+      </c>
+      <c r="E24" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F24" s="19" t="inlineStr">
+        <is>
+          <t>docker.socket permissions are correct (644 or 444).</t>
+        </is>
+      </c>
+      <c r="G24" s="19" t="inlineStr">
+        <is>
+          <t>chmod 644 /usr/lib/systemd/system/docker.socket</t>
+        </is>
+      </c>
+      <c r="H24" s="19" t="inlineStr">
+        <is>
+          <t>['0644', AnsibleUndefined(hint=None, obj={'exists': False}, name='mode'), '0644']</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="44" customHeight="1">
+      <c r="B25" s="21" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="inlineStr">
+        <is>
+          <t>Section 3 - Docker Daemon Configuration Files</t>
+        </is>
+      </c>
+      <c r="D25" s="22" t="inlineStr">
+        <is>
+          <t>Ensure that registry certificate file ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="E25" s="25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="F25" s="22" t="inlineStr">
+        <is>
+          <t>No registry certificates found in /etc/docker/certs.d.</t>
+        </is>
+      </c>
+      <c r="G25" s="22" t="inlineStr">
+        <is>
+          <t>chown root:root /etc/docker/certs.d/*/*.crt</t>
+        </is>
+      </c>
+      <c r="H25" s="22" t="inlineStr">
+        <is>
+          <t>0 certificate(s) found</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="44" customHeight="1">
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>3.6</t>
+        </is>
+      </c>
+      <c r="C26" s="19" t="inlineStr">
+        <is>
+          <t>Section 3 - Docker Daemon Configuration Files</t>
+        </is>
+      </c>
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>Ensure that registry certificate file permissions are set to 444 or more restrictively</t>
+        </is>
+      </c>
+      <c r="E26" s="25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="F26" s="19" t="inlineStr">
+        <is>
+          <t>No registry certificates found.</t>
+        </is>
+      </c>
+      <c r="G26" s="19" t="inlineStr">
+        <is>
+          <t>chmod 444 /etc/docker/certs.d/*/*.crt</t>
+        </is>
+      </c>
+      <c r="H26" s="19" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="44" customHeight="1">
+      <c r="B27" s="21" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
+      <c r="C27" s="22" t="inlineStr">
+        <is>
+          <t>Section 3 - Docker Daemon Configuration Files</t>
+        </is>
+      </c>
+      <c r="D27" s="22" t="inlineStr">
+        <is>
+          <t>Ensure that TLS CA certificate ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="E27" s="25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="F27" s="22" t="inlineStr">
+        <is>
+          <t>No TLS CA certificates found.</t>
+        </is>
+      </c>
+      <c r="G27" s="22" t="inlineStr">
+        <is>
+          <t>chown root:root /etc/docker/ca*.pem</t>
+        </is>
+      </c>
+      <c r="H27" s="22" t="inlineStr">
+        <is>
+          <t>0 CA certificate(s) found</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="44" customHeight="1">
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>3.8</t>
+        </is>
+      </c>
+      <c r="C28" s="19" t="inlineStr">
+        <is>
+          <t>Section 3 - Docker Daemon Configuration Files</t>
+        </is>
+      </c>
+      <c r="D28" s="19" t="inlineStr">
+        <is>
+          <t>Ensure that TLS CA certificate permissions are set to 444 or more restrictively</t>
+        </is>
+      </c>
+      <c r="E28" s="25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="F28" s="19" t="inlineStr">
+        <is>
+          <t>No TLS CA certificates found.</t>
+        </is>
+      </c>
+      <c r="G28" s="19" t="inlineStr">
+        <is>
+          <t>chmod 444 /etc/docker/ca*.pem</t>
+        </is>
+      </c>
+      <c r="H28" s="19" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="44" customHeight="1">
+      <c r="B29" s="21" t="inlineStr">
+        <is>
+          <t>3.9</t>
+        </is>
+      </c>
+      <c r="C29" s="22" t="inlineStr">
+        <is>
+          <t>Section 3 - Docker Daemon Configuration Files</t>
+        </is>
+      </c>
+      <c r="D29" s="22" t="inlineStr">
+        <is>
+          <t>Ensure that Docker server certificate file ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="E29" s="25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="F29" s="22" t="inlineStr">
+        <is>
+          <t>No Docker server certificates found.</t>
+        </is>
+      </c>
+      <c r="G29" s="22" t="inlineStr">
+        <is>
+          <t>chown root:root /etc/docker/server*.pem</t>
+        </is>
+      </c>
+      <c r="H29" s="22" t="inlineStr">
+        <is>
+          <t>0 server certificate(s) found</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="44" customHeight="1">
+      <c r="B30" s="18" t="inlineStr">
+        <is>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="C30" s="19" t="inlineStr">
+        <is>
+          <t>Section 3 - Docker Daemon Configuration Files</t>
+        </is>
+      </c>
+      <c r="D30" s="19" t="inlineStr">
+        <is>
+          <t>Ensure that Docker server certificate file permissions are set to 444 or more restrictively</t>
+        </is>
+      </c>
+      <c r="E30" s="25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="F30" s="19" t="inlineStr">
+        <is>
+          <t>No Docker server certificates found.</t>
+        </is>
+      </c>
+      <c r="G30" s="19" t="inlineStr">
+        <is>
+          <t>chmod 444 /etc/docker/server*.pem</t>
+        </is>
+      </c>
+      <c r="H30" s="19" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="44" customHeight="1">
+      <c r="B31" s="21" t="inlineStr">
+        <is>
+          <t>3.11</t>
+        </is>
+      </c>
+      <c r="C31" s="22" t="inlineStr">
+        <is>
+          <t>Section 3 - Docker Daemon Configuration Files</t>
+        </is>
+      </c>
+      <c r="D31" s="22" t="inlineStr">
+        <is>
+          <t>Ensure that the Docker server certificate key file ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="E31" s="25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="F31" s="22" t="inlineStr">
+        <is>
+          <t>No Docker server keys found.</t>
+        </is>
+      </c>
+      <c r="G31" s="22" t="inlineStr">
+        <is>
+          <t>chown root:root /etc/docker/server*.key</t>
+        </is>
+      </c>
+      <c r="H31" s="22" t="inlineStr">
+        <is>
+          <t>0 server key(s) found</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="44" customHeight="1">
+      <c r="B32" s="18" t="inlineStr">
+        <is>
+          <t>3.12</t>
+        </is>
+      </c>
+      <c r="C32" s="19" t="inlineStr">
+        <is>
+          <t>Section 3 - Docker Daemon Configuration Files</t>
+        </is>
+      </c>
+      <c r="D32" s="19" t="inlineStr">
+        <is>
+          <t>Ensure that the Docker server certificate key file permissions are set to 400</t>
+        </is>
+      </c>
+      <c r="E32" s="25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="F32" s="19" t="inlineStr">
+        <is>
+          <t>No Docker server keys found.</t>
+        </is>
+      </c>
+      <c r="G32" s="19" t="inlineStr">
+        <is>
+          <t>chmod 400 /etc/docker/server*.key</t>
+        </is>
+      </c>
+      <c r="H32" s="19" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="44" customHeight="1">
+      <c r="B33" s="21" t="inlineStr">
+        <is>
+          <t>3.13</t>
+        </is>
+      </c>
+      <c r="C33" s="22" t="inlineStr">
+        <is>
+          <t>Section 3 - Docker Daemon Configuration Files</t>
+        </is>
+      </c>
+      <c r="D33" s="22" t="inlineStr">
+        <is>
+          <t>Ensure that the Docker socket file ownership is set to root:docker</t>
+        </is>
+      </c>
+      <c r="E33" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F33" s="22" t="inlineStr">
+        <is>
+          <t>Docker socket ownership is correct (root:docker).</t>
+        </is>
+      </c>
+      <c r="G33" s="22" t="inlineStr">
+        <is>
+          <t>chown root:docker /var/run/docker.sock</t>
+        </is>
+      </c>
+      <c r="H33" s="22" t="inlineStr">
+        <is>
+          <t>root:docker</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="44" customHeight="1">
+      <c r="B34" s="18" t="inlineStr">
+        <is>
+          <t>3.14</t>
+        </is>
+      </c>
+      <c r="C34" s="19" t="inlineStr">
+        <is>
+          <t>Section 3 - Docker Daemon Configuration Files</t>
+        </is>
+      </c>
+      <c r="D34" s="19" t="inlineStr">
+        <is>
+          <t>Ensure that the Docker socket file permissions are set to 660 or more restrictively</t>
+        </is>
+      </c>
+      <c r="E34" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F34" s="19" t="inlineStr">
+        <is>
+          <t>Docker socket permissions are correct (660 or more restrictive).</t>
+        </is>
+      </c>
+      <c r="G34" s="19" t="inlineStr">
+        <is>
+          <t>chmod 660 /var/run/docker.sock</t>
+        </is>
+      </c>
+      <c r="H34" s="19" t="inlineStr">
+        <is>
+          <t>0660</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="44" customHeight="1">
+      <c r="B35" s="21" t="inlineStr">
+        <is>
+          <t>3.15</t>
+        </is>
+      </c>
+      <c r="C35" s="22" t="inlineStr">
+        <is>
+          <t>Section 3 - Docker Daemon Configuration Files</t>
+        </is>
+      </c>
+      <c r="D35" s="22" t="inlineStr">
+        <is>
+          <t>Ensure that the daemon.json file ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="E35" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F35" s="22" t="inlineStr">
+        <is>
+          <t>daemon.json ownership is correct (root:root).</t>
+        </is>
+      </c>
+      <c r="G35" s="22" t="inlineStr">
+        <is>
+          <t>chown root:root /etc/docker/daemon.json</t>
+        </is>
+      </c>
+      <c r="H35" s="22" t="inlineStr">
+        <is>
+          <t>root:root</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="44" customHeight="1">
+      <c r="B36" s="18" t="inlineStr">
+        <is>
+          <t>3.16</t>
+        </is>
+      </c>
+      <c r="C36" s="19" t="inlineStr">
+        <is>
+          <t>Section 3 - Docker Daemon Configuration Files</t>
+        </is>
+      </c>
+      <c r="D36" s="19" t="inlineStr">
+        <is>
+          <t>Ensure that daemon.json file permissions are set to 644 or more restrictive</t>
+        </is>
+      </c>
+      <c r="E36" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F36" s="19" t="inlineStr">
+        <is>
+          <t>daemon.json permissions are correct (644 or more restrictive).</t>
+        </is>
+      </c>
+      <c r="G36" s="19" t="inlineStr">
+        <is>
+          <t>chmod 644 /etc/docker/daemon.json</t>
+        </is>
+      </c>
+      <c r="H36" s="19" t="inlineStr">
+        <is>
+          <t>0644</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="44" customHeight="1">
+      <c r="B37" s="21" t="inlineStr">
+        <is>
+          <t>3.17</t>
+        </is>
+      </c>
+      <c r="C37" s="22" t="inlineStr">
+        <is>
+          <t>Section 3 - Docker Daemon Configuration Files</t>
+        </is>
+      </c>
+      <c r="D37" s="22" t="inlineStr">
+        <is>
+          <t>Ensure that the /etc/default/docker file ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="E37" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F37" s="22" t="inlineStr">
+        <is>
+          <t>/etc/default/docker ownership is correct (root:root).</t>
+        </is>
+      </c>
+      <c r="G37" s="22" t="inlineStr">
+        <is>
+          <t>chown root:root /etc/default/docker</t>
+        </is>
+      </c>
+      <c r="H37" s="22" t="inlineStr">
+        <is>
+          <t>root:root</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="44" customHeight="1">
+      <c r="B38" s="18" t="inlineStr">
+        <is>
+          <t>3.18</t>
+        </is>
+      </c>
+      <c r="C38" s="19" t="inlineStr">
+        <is>
+          <t>Section 3 - Docker Daemon Configuration Files</t>
+        </is>
+      </c>
+      <c r="D38" s="19" t="inlineStr">
+        <is>
+          <t>Ensure that the /etc/default/docker file permissions are set to 644 or more restrictively</t>
+        </is>
+      </c>
+      <c r="E38" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F38" s="19" t="inlineStr">
+        <is>
+          <t>/etc/default/docker permissions are correct (644 or more restrictive).</t>
+        </is>
+      </c>
+      <c r="G38" s="19" t="inlineStr">
+        <is>
+          <t>chmod 644 /etc/default/docker</t>
+        </is>
+      </c>
+      <c r="H38" s="19" t="inlineStr">
+        <is>
+          <t>0644</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="44" customHeight="1">
+      <c r="B39" s="21" t="inlineStr">
+        <is>
+          <t>3.19</t>
+        </is>
+      </c>
+      <c r="C39" s="22" t="inlineStr">
+        <is>
+          <t>Section 3 - Docker Daemon Configuration Files</t>
+        </is>
+      </c>
+      <c r="D39" s="22" t="inlineStr">
+        <is>
+          <t>Ensure that the /etc/sysconfig/docker file permissions are set to 644 or more restrictively</t>
+        </is>
+      </c>
+      <c r="E39" s="25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="F39" s="22" t="inlineStr">
+        <is>
+          <t>/etc/sysconfig/docker does not exist.</t>
+        </is>
+      </c>
+      <c r="G39" s="22" t="inlineStr">
+        <is>
+          <t>chmod 644 /etc/sysconfig/docker</t>
+        </is>
+      </c>
+      <c r="H39" s="22" t="inlineStr">
+        <is>
+          <t>File does not exist</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="44" customHeight="1">
+      <c r="B40" s="18" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="C40" s="19" t="inlineStr">
+        <is>
+          <t>Section 3 - Docker Daemon Configuration Files</t>
+        </is>
+      </c>
+      <c r="D40" s="19" t="inlineStr">
+        <is>
+          <t>Ensure that the /etc/sysconfig/docker file ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="E40" s="25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="F40" s="19" t="inlineStr">
+        <is>
+          <t>/etc/sysconfig/docker does not exist.</t>
+        </is>
+      </c>
+      <c r="G40" s="19" t="inlineStr">
+        <is>
+          <t>chown root:root /etc/sysconfig/docker</t>
+        </is>
+      </c>
+      <c r="H40" s="19" t="inlineStr">
+        <is>
+          <t>File does not exist</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="44" customHeight="1">
+      <c r="B41" s="21" t="inlineStr">
+        <is>
+          <t>3.21</t>
+        </is>
+      </c>
+      <c r="C41" s="22" t="inlineStr">
+        <is>
+          <t>Section 3 - Docker Daemon Configuration Files</t>
+        </is>
+      </c>
+      <c r="D41" s="22" t="inlineStr">
+        <is>
+          <t>Ensure that the Containerd socket file ownership is set to root:root</t>
+        </is>
+      </c>
+      <c r="E41" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F41" s="22" t="inlineStr">
+        <is>
+          <t>containerd socket ownership is correct (root:root).</t>
+        </is>
+      </c>
+      <c r="G41" s="22" t="inlineStr">
+        <is>
+          <t>chown root:root /run/containerd/containerd.sock</t>
+        </is>
+      </c>
+      <c r="H41" s="22" t="inlineStr">
+        <is>
+          <t>root:root</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="44" customHeight="1">
+      <c r="B42" s="18" t="inlineStr">
+        <is>
+          <t>3.22</t>
+        </is>
+      </c>
+      <c r="C42" s="19" t="inlineStr">
+        <is>
+          <t>Section 3 - Docker Daemon Configuration Files</t>
+        </is>
+      </c>
+      <c r="D42" s="19" t="inlineStr">
+        <is>
+          <t>Ensure that the Containerd socket file permissions are set to 660 or more restrictively</t>
+        </is>
+      </c>
+      <c r="E42" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F42" s="19" t="inlineStr">
+        <is>
+          <t>containerd socket permissions are correct (660 or more restrictive).</t>
+        </is>
+      </c>
+      <c r="G42" s="19" t="inlineStr">
+        <is>
+          <t>chmod 660 /run/containerd/containerd.sock</t>
+        </is>
+      </c>
+      <c r="H42" s="19" t="inlineStr">
+        <is>
+          <t>0660</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:H10"/>
+  <autoFilter ref="B1:H42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1515,7 +3540,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3">
@@ -1525,7 +3550,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -1535,7 +3560,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -1545,7 +3570,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix the format + all excel file + LOL done + fix folder
</commit_message>
<xml_diff>
--- a/audit/docker_benchmark_reports/192.168.1.8_section2_3.xlsx
+++ b/audit/docker_benchmark_reports/192.168.1.8_section2_3.xlsx
@@ -796,7 +796,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Daemon Configuration &amp; Files  |  Host: Docker-2204-DA-AUTO  |  Docker:   |  OS: Ubuntu 22.04  |  2026-05-18T05:21:16Z</t>
+          <t>Daemon Configuration &amp; Files  |  Host: Docker-2204-DA-AUTO  |  Docker: 29.4.3  |  OS: Ubuntu 22.04  |  2026-05-18T05:37:57Z</t>
         </is>
       </c>
     </row>
@@ -828,10 +828,10 @@
         <v>41</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>13</v>
@@ -840,7 +840,7 @@
     <row r="8" ht="28" customHeight="1">
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Compliance:  ███████████░░░░░░░░░  56.1%  (23 / 41 passed)</t>
+          <t xml:space="preserve">  Compliance:  ████████████░░░░░░░░  61.0%  (25 / 41 passed)</t>
         </is>
       </c>
     </row>
@@ -921,14 +921,14 @@
           <t>Ensure the logging level is set to 'info'</t>
         </is>
       </c>
-      <c r="F13" s="15" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>Logging level is set to info.</t>
+          <t>Logging level is NOT set to info. Default may be too verbose or not verbose enough.</t>
         </is>
       </c>
     </row>
@@ -994,7 +994,7 @@
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>Storage driver is  (not aufs).</t>
+          <t>Storage driver is overlay2 (not aufs).</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
-          <t>Storage driver is  (not devicemapper).</t>
+          <t>Storage driver is overlay2 (not devicemapper).</t>
         </is>
       </c>
     </row>
@@ -1031,14 +1031,14 @@
           <t>Ensure TLS authentication for Docker daemon is configured</t>
         </is>
       </c>
-      <c r="F18" s="15" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>TLS authentication is enabled with tls and tlsverify configured.</t>
+          <t>TLS authentication is NOT configured. Docker API communications may be unencrypted.</t>
         </is>
       </c>
     </row>
@@ -1053,14 +1053,14 @@
           <t>Ensure the default ulimit is configured appropriately</t>
         </is>
       </c>
-      <c r="F19" s="15" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>Default ulimits are configured in daemon.json.</t>
+          <t>Default ulimits are NOT configured. Containers may exhaust system resources.</t>
         </is>
       </c>
     </row>
@@ -1104,8 +1104,7 @@
       </c>
       <c r="G21" s="11" t="inlineStr">
         <is>
-          <t>Cgroup driver: 
-INFO</t>
+          <t>Cgroup driver: systemd</t>
         </is>
       </c>
     </row>
@@ -1142,14 +1141,14 @@
           <t>Ensure that authorization for Docker client commands is enabled</t>
         </is>
       </c>
-      <c r="F23" s="16" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="F23" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G23" s="11" t="inlineStr">
         <is>
-          <t>Authorization plugins are NOT configured. Docker commands are not audited/controlled.</t>
+          <t>Authorization plugins are configured in daemon.json.</t>
         </is>
       </c>
     </row>
@@ -1164,14 +1163,14 @@
           <t>Ensure centralized and remote logging is configured</t>
         </is>
       </c>
-      <c r="F24" s="16" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="F24" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
-          <t>Centralized logging is NOT configured. Logs may be lost if host fails.</t>
+          <t>Centralized logging driver is configured.</t>
         </is>
       </c>
     </row>
@@ -1186,14 +1185,14 @@
           <t>Ensure containers are restricted from acquiring new privileges</t>
         </is>
       </c>
-      <c r="F25" s="16" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="F25" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G25" s="11" t="inlineStr">
         <is>
-          <t>no-new-privileges is NOT set. Containers can escalate privileges via setuid binaries.</t>
+          <t>no-new-privileges is set to true in daemon.json.</t>
         </is>
       </c>
     </row>
@@ -1208,14 +1207,14 @@
           <t>Ensure live restore is enabled</t>
         </is>
       </c>
-      <c r="F26" s="16" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="F26" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
-          <t>Live restore is NOT enabled. Containers stop when Docker daemon restarts.</t>
+          <t>Live restore is enabled. Containers survive Docker daemon restarts.</t>
         </is>
       </c>
     </row>
@@ -1230,14 +1229,14 @@
           <t>Ensure Userland Proxy is Disabled</t>
         </is>
       </c>
-      <c r="F27" s="16" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="F27" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G27" s="11" t="inlineStr">
         <is>
-          <t>Userland proxy is enabled. This can cause performance issues and port conflicts.</t>
+          <t>Userland proxy is disabled. Docker uses kernel NAT for better performance.</t>
         </is>
       </c>
     </row>
@@ -2081,7 +2080,7 @@
       </c>
       <c r="H3" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "icc": false,</t>
+          <t>{"icc": false, "userns-remap": "default", "log-driver": "syslog", "log-opts": {"syslog-address": "udp://127.0.0.1:514", "syslog-facility": "daemon", "tag": "docker/{{.Name}}"}, "no-new-privileges": true, "live-restore": true, "userland-proxy": false, "authorization-plugins": ["opa-docker-authz"]}</t>
         </is>
       </c>
     </row>
@@ -2101,14 +2100,14 @@
           <t>Ensure the logging level is set to 'info'</t>
         </is>
       </c>
-      <c r="E4" s="23" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="E4" s="24" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="F4" s="19" t="inlineStr">
         <is>
-          <t>Logging level is set to info.</t>
+          <t>Logging level is NOT set to info. Default may be too verbose or not verbose enough.</t>
         </is>
       </c>
       <c r="G4" s="19" t="inlineStr">
@@ -2116,11 +2115,7 @@
           <t>Add "log-level": "info" to /etc/docker/daemon.json</t>
         </is>
       </c>
-      <c r="H4" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    "log-level": "info",</t>
-        </is>
-      </c>
+      <c r="H4" s="19" t="inlineStr"/>
     </row>
     <row r="5" ht="44" customHeight="1">
       <c r="B5" s="21" t="inlineStr">
@@ -2155,7 +2150,7 @@
       </c>
       <c r="H5" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "iptables": true,</t>
+          <t>INFO: Default is true</t>
         </is>
       </c>
     </row>
@@ -2219,7 +2214,7 @@
       </c>
       <c r="F7" s="22" t="inlineStr">
         <is>
-          <t>Storage driver is  (not aufs).</t>
+          <t>Storage driver is overlay2 (not aufs).</t>
         </is>
       </c>
       <c r="G7" s="22" t="inlineStr">
@@ -2227,7 +2222,11 @@
           <t>Change storage driver to overlay2 in /etc/docker/daemon.json: {"storage-driver": "overlay2"}</t>
         </is>
       </c>
-      <c r="H7" s="22" t="inlineStr"/>
+      <c r="H7" s="22" t="inlineStr">
+        <is>
+          <t>overlay2</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="44" customHeight="1">
       <c r="B8" s="18" t="inlineStr">
@@ -2252,7 +2251,7 @@
       </c>
       <c r="F8" s="19" t="inlineStr">
         <is>
-          <t>Storage driver is  (not devicemapper).</t>
+          <t>Storage driver is overlay2 (not devicemapper).</t>
         </is>
       </c>
       <c r="G8" s="19" t="inlineStr">
@@ -2260,7 +2259,11 @@
           <t>Change storage driver to overlay2 in /etc/docker/daemon.json: {"storage-driver": "overlay2"}</t>
         </is>
       </c>
-      <c r="H8" s="19" t="inlineStr"/>
+      <c r="H8" s="19" t="inlineStr">
+        <is>
+          <t>overlay2</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="44" customHeight="1">
       <c r="B9" s="21" t="inlineStr">
@@ -2278,14 +2281,14 @@
           <t>Ensure TLS authentication for Docker daemon is configured</t>
         </is>
       </c>
-      <c r="E9" s="23" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="F9" s="22" t="inlineStr">
         <is>
-          <t>TLS authentication is enabled with tls and tlsverify configured.</t>
+          <t>TLS authentication is NOT configured. Docker API communications may be unencrypted.</t>
         </is>
       </c>
       <c r="G9" s="22" t="inlineStr">
@@ -2293,12 +2296,7 @@
           <t>Configure TLS in /etc/docker/daemon.json with "tls": true and "tlsverify": true. Ensure CA, server cert, and server key paths are correctly specified.</t>
         </is>
       </c>
-      <c r="H9" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    "tls": true,
-    "tlsverify": true,</t>
-        </is>
-      </c>
+      <c r="H9" s="22" t="inlineStr"/>
     </row>
     <row r="10" ht="44" customHeight="1">
       <c r="B10" s="18" t="inlineStr">
@@ -2316,14 +2314,14 @@
           <t>Ensure the default ulimit is configured appropriately</t>
         </is>
       </c>
-      <c r="E10" s="23" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="E10" s="24" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="F10" s="19" t="inlineStr">
         <is>
-          <t>Default ulimits are configured in daemon.json.</t>
+          <t>Default ulimits are NOT configured. Containers may exhaust system resources.</t>
         </is>
       </c>
       <c r="G10" s="19" t="inlineStr">
@@ -2331,11 +2329,7 @@
           <t>Configure default ulimits in /etc/docker/daemon.json: {"default-ulimits": {"nofile": {"Hard": 64000, "Name": "nofile", "Soft": 64000}}}</t>
         </is>
       </c>
-      <c r="H10" s="19" t="inlineStr">
-        <is>
-          <t>"default-ulimits": {</t>
-        </is>
-      </c>
+      <c r="H10" s="19" t="inlineStr"/>
     </row>
     <row r="11" ht="44" customHeight="1">
       <c r="B11" s="21" t="inlineStr">
@@ -2370,7 +2364,7 @@
       </c>
       <c r="H11" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "userns-remap": "default",</t>
+          <t>{"icc": false, "userns-remap": "default", "log-driver": "syslog", "log-opts": {"syslog-address": "udp://127.0.0.1:514", "syslog-facility": "daemon", "tag": "docker/{{.Name}}"}, "no-new-privileges": true, "live-restore": true, "userland-proxy": false, "authorization-plugins": ["opa-docker-authz"]}</t>
         </is>
       </c>
     </row>
@@ -2397,8 +2391,7 @@
       </c>
       <c r="F12" s="19" t="inlineStr">
         <is>
-          <t>Cgroup driver: 
-INFO</t>
+          <t>Cgroup driver: systemd</t>
         </is>
       </c>
       <c r="G12" s="19" t="inlineStr">
@@ -2408,8 +2401,7 @@
       </c>
       <c r="H12" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">
-INFO</t>
+          <t>systemd</t>
         </is>
       </c>
     </row>
@@ -2466,14 +2458,14 @@
           <t>Ensure that authorization for Docker client commands is enabled</t>
         </is>
       </c>
-      <c r="E14" s="24" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E14" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F14" s="19" t="inlineStr">
         <is>
-          <t>Authorization plugins are NOT configured. Docker commands are not audited/controlled.</t>
+          <t>Authorization plugins are configured in daemon.json.</t>
         </is>
       </c>
       <c r="G14" s="19" t="inlineStr">
@@ -2481,7 +2473,11 @@
           <t>Add authorization plugins to /etc/docker/daemon.json: {"authorization-plugins": ["openpolicyagent/opa-docker-authz"]}</t>
         </is>
       </c>
-      <c r="H14" s="19" t="inlineStr"/>
+      <c r="H14" s="19" t="inlineStr">
+        <is>
+          <t>{"icc": false, "userns-remap": "default", "log-driver": "syslog", "log-opts": {"syslog-address": "udp://127.0.0.1:514", "syslog-facility": "daemon", "tag": "docker/{{.Name}}"}, "no-new-privileges": true, "live-restore": true, "userland-proxy": false, "authorization-plugins": ["opa-docker-authz"]}</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="44" customHeight="1">
       <c r="B15" s="21" t="inlineStr">
@@ -2499,14 +2495,14 @@
           <t>Ensure centralized and remote logging is configured</t>
         </is>
       </c>
-      <c r="E15" s="24" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E15" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F15" s="22" t="inlineStr">
         <is>
-          <t>Centralized logging is NOT configured. Logs may be lost if host fails.</t>
+          <t>Centralized logging driver is configured.</t>
         </is>
       </c>
       <c r="G15" s="22" t="inlineStr">
@@ -2514,7 +2510,11 @@
           <t>Configure a centralized logging driver in /etc/docker/daemon.json: {"log-driver": "syslog", "log-opts": {"syslog-address": "tcp://192.168.0.42:12345"}}</t>
         </is>
       </c>
-      <c r="H15" s="22" t="inlineStr"/>
+      <c r="H15" s="22" t="inlineStr">
+        <is>
+          <t>{"icc": false, "userns-remap": "default", "log-driver": "syslog", "log-opts": {"syslog-address": "udp://127.0.0.1:514", "syslog-facility": "daemon", "tag": "docker/{{.Name}}"}, "no-new-privileges": true, "live-restore": true, "userland-proxy": false, "authorization-plugins": ["opa-docker-authz"]}</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="44" customHeight="1">
       <c r="B16" s="18" t="inlineStr">
@@ -2532,14 +2532,14 @@
           <t>Ensure containers are restricted from acquiring new privileges</t>
         </is>
       </c>
-      <c r="E16" s="24" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E16" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F16" s="19" t="inlineStr">
         <is>
-          <t>no-new-privileges is NOT set. Containers can escalate privileges via setuid binaries.</t>
+          <t>no-new-privileges is set to true in daemon.json.</t>
         </is>
       </c>
       <c r="G16" s="19" t="inlineStr">
@@ -2547,7 +2547,11 @@
           <t>Add "no-new-privileges": true to /etc/docker/daemon.json</t>
         </is>
       </c>
-      <c r="H16" s="19" t="inlineStr"/>
+      <c r="H16" s="19" t="inlineStr">
+        <is>
+          <t>{"icc": false, "userns-remap": "default", "log-driver": "syslog", "log-opts": {"syslog-address": "udp://127.0.0.1:514", "syslog-facility": "daemon", "tag": "docker/{{.Name}}"}, "no-new-privileges": true, "live-restore": true, "userland-proxy": false, "authorization-plugins": ["opa-docker-authz"]}</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="44" customHeight="1">
       <c r="B17" s="21" t="inlineStr">
@@ -2565,14 +2569,14 @@
           <t>Ensure live restore is enabled</t>
         </is>
       </c>
-      <c r="E17" s="24" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E17" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F17" s="22" t="inlineStr">
         <is>
-          <t>Live restore is NOT enabled. Containers stop when Docker daemon restarts.</t>
+          <t>Live restore is enabled. Containers survive Docker daemon restarts.</t>
         </is>
       </c>
       <c r="G17" s="22" t="inlineStr">
@@ -2580,7 +2584,11 @@
           <t>Add "live-restore": true to /etc/docker/daemon.json</t>
         </is>
       </c>
-      <c r="H17" s="22" t="inlineStr"/>
+      <c r="H17" s="22" t="inlineStr">
+        <is>
+          <t>{"icc": false, "userns-remap": "default", "log-driver": "syslog", "log-opts": {"syslog-address": "udp://127.0.0.1:514", "syslog-facility": "daemon", "tag": "docker/{{.Name}}"}, "no-new-privileges": true, "live-restore": true, "userland-proxy": false, "authorization-plugins": ["opa-docker-authz"]}</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="44" customHeight="1">
       <c r="B18" s="18" t="inlineStr">
@@ -2598,14 +2606,14 @@
           <t>Ensure Userland Proxy is Disabled</t>
         </is>
       </c>
-      <c r="E18" s="24" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E18" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F18" s="19" t="inlineStr">
         <is>
-          <t>Userland proxy is enabled. This can cause performance issues and port conflicts.</t>
+          <t>Userland proxy is disabled. Docker uses kernel NAT for better performance.</t>
         </is>
       </c>
       <c r="G18" s="19" t="inlineStr">
@@ -2613,7 +2621,11 @@
           <t>Add "userland-proxy": false to /etc/docker/daemon.json</t>
         </is>
       </c>
-      <c r="H18" s="19" t="inlineStr"/>
+      <c r="H18" s="19" t="inlineStr">
+        <is>
+          <t>{"icc": false, "userns-remap": "default", "log-driver": "syslog", "log-opts": {"syslog-address": "udp://127.0.0.1:514", "syslog-facility": "daemon", "tag": "docker/{{.Name}}"}, "no-new-privileges": true, "live-restore": true, "userland-proxy": false, "authorization-plugins": ["opa-docker-authz"]}</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="44" customHeight="1">
       <c r="B19" s="21" t="inlineStr">
@@ -3540,7 +3552,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3">
@@ -3550,7 +3562,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">

</xml_diff>